<commit_message>
Seed PUMA India discovery queue
</commit_message>
<xml_diff>
--- a/outputs/catalog-intake-template/runwise-india-shoe-catalog-intake.xlsx
+++ b/outputs/catalog-intake-template/runwise-india-shoe-catalog-intake.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog Intake" sheetId="1" r:id="R1fc7d9a123e947aa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; Lists" sheetId="2" r:id="Rbff95772b56c4869"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalog Intake" sheetId="1" r:id="Rff52083d92674466"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide &amp; Lists" sheetId="2" r:id="Rf0912229f73b4156"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PUMA Discovery" sheetId="3" r:id="R1662d5fd238f4619"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -212,7 +213,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="80">
+  <x:cellXfs count="88">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -399,11 +400,35 @@
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
   </x:cellStyles>
-  <x:dxfs count="3">
+  <x:dxfs count="5">
     <x:dxf>
       <x:font>
         <x:b/>
@@ -420,6 +445,18 @@
       <x:font>
         <x:b/>
         <x:color rgb="FF9B2C2C"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF276749"/>
+      </x:font>
+    </x:dxf>
+    <x:dxf>
+      <x:font>
+        <x:b/>
+        <x:color rgb="FF8A5A00"/>
       </x:font>
     </x:dxf>
   </x:dxfs>
@@ -5151,4 +5188,687 @@
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="12" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="33" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="12" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="19" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="49" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="21" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="15" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="34" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="30" customHeight="1">
+      <x:c r="A1" s="65" t="str">
+        <x:v>PUMA India · NITRO discovery queue</x:v>
+      </x:c>
+      <x:c r="B1" s="65"/>
+      <x:c r="C1" s="65"/>
+      <x:c r="D1" s="65"/>
+      <x:c r="E1" s="65"/>
+      <x:c r="F1" s="65"/>
+      <x:c r="G1" s="65"/>
+      <x:c r="H1" s="65"/>
+      <x:c r="I1" s="65"/>
+      <x:c r="J1" s="65"/>
+    </x:row>
+    <x:row r="2" ht="30" customHeight="1">
+      <x:c r="A2" s="7" t="str">
+        <x:v>Official collection listing discovered 18 distinct model / gender candidates. These are not live catalog records until product-page specs and a direct URL are verified.</x:v>
+      </x:c>
+      <x:c r="B2" s="7"/>
+      <x:c r="C2" s="7"/>
+      <x:c r="D2" s="7"/>
+      <x:c r="E2" s="7"/>
+      <x:c r="F2" s="7"/>
+      <x:c r="G2" s="7"/>
+      <x:c r="H2" s="7"/>
+      <x:c r="I2" s="7"/>
+      <x:c r="J2" s="7"/>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="81" t="str">
+        <x:v>brand</x:v>
+      </x:c>
+      <x:c r="B4" s="81" t="str">
+        <x:v>model</x:v>
+      </x:c>
+      <x:c r="C4" s="81" t="str">
+        <x:v>gender</x:v>
+      </x:c>
+      <x:c r="D4" s="81" t="str">
+        <x:v>category</x:v>
+      </x:c>
+      <x:c r="E4" s="81" t="str">
+        <x:v>observed price (INR)</x:v>
+      </x:c>
+      <x:c r="F4" s="81" t="str">
+        <x:v>observed MRP (INR)</x:v>
+      </x:c>
+      <x:c r="G4" s="81" t="str">
+        <x:v>collection source</x:v>
+      </x:c>
+      <x:c r="H4" s="81" t="str">
+        <x:v>status</x:v>
+      </x:c>
+      <x:c r="I4" s="81" t="str">
+        <x:v>retrieved on</x:v>
+      </x:c>
+      <x:c r="J4" s="81" t="str">
+        <x:v>next action</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="37" t="str">
+        <x:v>PUMA</x:v>
+      </x:c>
+      <x:c r="B5" s="37" t="str">
+        <x:v>MagMax NITRO 2</x:v>
+      </x:c>
+      <x:c r="C5" s="37" t="str">
+        <x:v>men</x:v>
+      </x:c>
+      <x:c r="D5" s="37" t="str">
+        <x:v>road</x:v>
+      </x:c>
+      <x:c r="E5" s="82" t="n">
+        <x:v>16999</x:v>
+      </x:c>
+      <x:c r="F5" s="82" t="n">
+        <x:v>16999</x:v>
+      </x:c>
+      <x:c r="G5" s="37" t="str">
+        <x:v>https://in.puma.com/in/en/sports/sports-running/nitro-collection</x:v>
+      </x:c>
+      <x:c r="H5" s="37" t="str">
+        <x:v>candidate</x:v>
+      </x:c>
+      <x:c r="I5" s="85" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="J5" s="37" t="str">
+        <x:f>IF(H5="already_in_catalog","Compare price and source","Open product page; complete specs")</x:f>
+        <x:v>Open product page; complete specs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="38" t="str">
+        <x:v>PUMA</x:v>
+      </x:c>
+      <x:c r="B6" s="38" t="str">
+        <x:v>MagMax NITRO 2</x:v>
+      </x:c>
+      <x:c r="C6" s="38" t="str">
+        <x:v>women</x:v>
+      </x:c>
+      <x:c r="D6" s="38" t="str">
+        <x:v>road</x:v>
+      </x:c>
+      <x:c r="E6" s="83" t="n">
+        <x:v>16999</x:v>
+      </x:c>
+      <x:c r="F6" s="83" t="n">
+        <x:v>16999</x:v>
+      </x:c>
+      <x:c r="G6" s="38" t="str">
+        <x:v>https://in.puma.com/in/en/sports/sports-running/nitro-collection</x:v>
+      </x:c>
+      <x:c r="H6" s="38" t="str">
+        <x:v>candidate</x:v>
+      </x:c>
+      <x:c r="I6" s="86" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="J6" s="38" t="str">
+        <x:f>IF(H6="already_in_catalog","Compare price and source","Open product page; complete specs")</x:f>
+        <x:v>Open product page; complete specs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="38" t="str">
+        <x:v>PUMA</x:v>
+      </x:c>
+      <x:c r="B7" s="38" t="str">
+        <x:v>PUMA x HYROX Velocity NITRO 5</x:v>
+      </x:c>
+      <x:c r="C7" s="38" t="str">
+        <x:v>men</x:v>
+      </x:c>
+      <x:c r="D7" s="38" t="str">
+        <x:v>road</x:v>
+      </x:c>
+      <x:c r="E7" s="83" t="n">
+        <x:v>12999</x:v>
+      </x:c>
+      <x:c r="F7" s="83" t="n">
+        <x:v>12999</x:v>
+      </x:c>
+      <x:c r="G7" s="38" t="str">
+        <x:v>https://in.puma.com/in/en/sports/sports-running/nitro-collection</x:v>
+      </x:c>
+      <x:c r="H7" s="38" t="str">
+        <x:v>candidate</x:v>
+      </x:c>
+      <x:c r="I7" s="86" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="J7" s="38" t="str">
+        <x:f>IF(H7="already_in_catalog","Compare price and source","Open product page; complete specs")</x:f>
+        <x:v>Open product page; complete specs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="38" t="str">
+        <x:v>PUMA</x:v>
+      </x:c>
+      <x:c r="B8" s="38" t="str">
+        <x:v>PUMA x HYROX Velocity NITRO 5</x:v>
+      </x:c>
+      <x:c r="C8" s="38" t="str">
+        <x:v>women</x:v>
+      </x:c>
+      <x:c r="D8" s="38" t="str">
+        <x:v>road</x:v>
+      </x:c>
+      <x:c r="E8" s="83" t="n">
+        <x:v>12999</x:v>
+      </x:c>
+      <x:c r="F8" s="83" t="n">
+        <x:v>12999</x:v>
+      </x:c>
+      <x:c r="G8" s="38" t="str">
+        <x:v>https://in.puma.com/in/en/sports/sports-running/nitro-collection</x:v>
+      </x:c>
+      <x:c r="H8" s="38" t="str">
+        <x:v>candidate</x:v>
+      </x:c>
+      <x:c r="I8" s="86" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="J8" s="38" t="str">
+        <x:f>IF(H8="already_in_catalog","Compare price and source","Open product page; complete specs")</x:f>
+        <x:v>Open product page; complete specs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="38" t="str">
+        <x:v>PUMA</x:v>
+      </x:c>
+      <x:c r="B9" s="38" t="str">
+        <x:v>PUMA x HYROX Deviate NITRO Elite 4</x:v>
+      </x:c>
+      <x:c r="C9" s="38" t="str">
+        <x:v>men</x:v>
+      </x:c>
+      <x:c r="D9" s="38" t="str">
+        <x:v>road</x:v>
+      </x:c>
+      <x:c r="E9" s="83" t="n">
+        <x:v>21999</x:v>
+      </x:c>
+      <x:c r="F9" s="83" t="n">
+        <x:v>21999</x:v>
+      </x:c>
+      <x:c r="G9" s="38" t="str">
+        <x:v>https://in.puma.com/in/en/sports/sports-running/nitro-collection</x:v>
+      </x:c>
+      <x:c r="H9" s="38" t="str">
+        <x:v>candidate</x:v>
+      </x:c>
+      <x:c r="I9" s="86" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="J9" s="38" t="str">
+        <x:f>IF(H9="already_in_catalog","Compare price and source","Open product page; complete specs")</x:f>
+        <x:v>Open product page; complete specs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="38" t="str">
+        <x:v>PUMA</x:v>
+      </x:c>
+      <x:c r="B10" s="38" t="str">
+        <x:v>PUMA x HYROX Deviate NITRO Elite 4</x:v>
+      </x:c>
+      <x:c r="C10" s="38" t="str">
+        <x:v>women</x:v>
+      </x:c>
+      <x:c r="D10" s="38" t="str">
+        <x:v>road</x:v>
+      </x:c>
+      <x:c r="E10" s="83" t="n">
+        <x:v>21999</x:v>
+      </x:c>
+      <x:c r="F10" s="83" t="n">
+        <x:v>21999</x:v>
+      </x:c>
+      <x:c r="G10" s="38" t="str">
+        <x:v>https://in.puma.com/in/en/sports/sports-running/nitro-collection</x:v>
+      </x:c>
+      <x:c r="H10" s="38" t="str">
+        <x:v>candidate</x:v>
+      </x:c>
+      <x:c r="I10" s="86" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="J10" s="38" t="str">
+        <x:f>IF(H10="already_in_catalog","Compare price and source","Open product page; complete specs")</x:f>
+        <x:v>Open product page; complete specs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="38" t="str">
+        <x:v>PUMA</x:v>
+      </x:c>
+      <x:c r="B11" s="38" t="str">
+        <x:v>Electrify NITRO 4</x:v>
+      </x:c>
+      <x:c r="C11" s="38" t="str">
+        <x:v>men</x:v>
+      </x:c>
+      <x:c r="D11" s="38" t="str">
+        <x:v>road</x:v>
+      </x:c>
+      <x:c r="E11" s="83" t="n">
+        <x:v>6299</x:v>
+      </x:c>
+      <x:c r="F11" s="83" t="n">
+        <x:v>8999</x:v>
+      </x:c>
+      <x:c r="G11" s="38" t="str">
+        <x:v>https://in.puma.com/in/en/sports/sports-running/nitro-collection</x:v>
+      </x:c>
+      <x:c r="H11" s="38" t="str">
+        <x:v>candidate</x:v>
+      </x:c>
+      <x:c r="I11" s="86" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="J11" s="38" t="str">
+        <x:f>IF(H11="already_in_catalog","Compare price and source","Open product page; complete specs")</x:f>
+        <x:v>Open product page; complete specs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="38" t="str">
+        <x:v>PUMA</x:v>
+      </x:c>
+      <x:c r="B12" s="38" t="str">
+        <x:v>Liberate NITRO 2</x:v>
+      </x:c>
+      <x:c r="C12" s="38" t="str">
+        <x:v>women</x:v>
+      </x:c>
+      <x:c r="D12" s="38" t="str">
+        <x:v>road</x:v>
+      </x:c>
+      <x:c r="E12" s="83" t="n">
+        <x:v>7199</x:v>
+      </x:c>
+      <x:c r="F12" s="83" t="n">
+        <x:v>11999</x:v>
+      </x:c>
+      <x:c r="G12" s="38" t="str">
+        <x:v>https://in.puma.com/in/en/sports/sports-running/nitro-collection</x:v>
+      </x:c>
+      <x:c r="H12" s="38" t="str">
+        <x:v>candidate</x:v>
+      </x:c>
+      <x:c r="I12" s="86" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="J12" s="38" t="str">
+        <x:f>IF(H12="already_in_catalog","Compare price and source","Open product page; complete specs")</x:f>
+        <x:v>Open product page; complete specs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="38" t="str">
+        <x:v>PUMA</x:v>
+      </x:c>
+      <x:c r="B13" s="38" t="str">
+        <x:v>PUMA x HYROX Deviate NITRO 4</x:v>
+      </x:c>
+      <x:c r="C13" s="38" t="str">
+        <x:v>men</x:v>
+      </x:c>
+      <x:c r="D13" s="38" t="str">
+        <x:v>road</x:v>
+      </x:c>
+      <x:c r="E13" s="83" t="n">
+        <x:v>16999</x:v>
+      </x:c>
+      <x:c r="F13" s="83" t="n">
+        <x:v>16999</x:v>
+      </x:c>
+      <x:c r="G13" s="38" t="str">
+        <x:v>https://in.puma.com/in/en/sports/sports-running/nitro-collection</x:v>
+      </x:c>
+      <x:c r="H13" s="38" t="str">
+        <x:v>candidate</x:v>
+      </x:c>
+      <x:c r="I13" s="86" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="J13" s="38" t="str">
+        <x:f>IF(H13="already_in_catalog","Compare price and source","Open product page; complete specs")</x:f>
+        <x:v>Open product page; complete specs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14">
+      <x:c r="A14" s="38" t="str">
+        <x:v>PUMA</x:v>
+      </x:c>
+      <x:c r="B14" s="38" t="str">
+        <x:v>PUMA x HYROX Deviate NITRO 4</x:v>
+      </x:c>
+      <x:c r="C14" s="38" t="str">
+        <x:v>women</x:v>
+      </x:c>
+      <x:c r="D14" s="38" t="str">
+        <x:v>road</x:v>
+      </x:c>
+      <x:c r="E14" s="83" t="n">
+        <x:v>16999</x:v>
+      </x:c>
+      <x:c r="F14" s="83" t="n">
+        <x:v>16999</x:v>
+      </x:c>
+      <x:c r="G14" s="38" t="str">
+        <x:v>https://in.puma.com/in/en/sports/sports-running/nitro-collection</x:v>
+      </x:c>
+      <x:c r="H14" s="38" t="str">
+        <x:v>candidate</x:v>
+      </x:c>
+      <x:c r="I14" s="86" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="J14" s="38" t="str">
+        <x:f>IF(H14="already_in_catalog","Compare price and source","Open product page; complete specs")</x:f>
+        <x:v>Open product page; complete specs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" s="38" t="str">
+        <x:v>PUMA</x:v>
+      </x:c>
+      <x:c r="B15" s="38" t="str">
+        <x:v>FAST-R NITRO Elite 3</x:v>
+      </x:c>
+      <x:c r="C15" s="38" t="str">
+        <x:v>women</x:v>
+      </x:c>
+      <x:c r="D15" s="38" t="str">
+        <x:v>road</x:v>
+      </x:c>
+      <x:c r="E15" s="83" t="n">
+        <x:v>23999</x:v>
+      </x:c>
+      <x:c r="F15" s="83" t="n">
+        <x:v>23999</x:v>
+      </x:c>
+      <x:c r="G15" s="38" t="str">
+        <x:v>https://in.puma.com/in/en/sports/sports-running/nitro-collection</x:v>
+      </x:c>
+      <x:c r="H15" s="38" t="str">
+        <x:v>candidate</x:v>
+      </x:c>
+      <x:c r="I15" s="86" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="J15" s="38" t="str">
+        <x:f>IF(H15="already_in_catalog","Compare price and source","Open product page; complete specs")</x:f>
+        <x:v>Open product page; complete specs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="38" t="str">
+        <x:v>PUMA</x:v>
+      </x:c>
+      <x:c r="B16" s="38" t="str">
+        <x:v>Deviate NITRO Elite 3</x:v>
+      </x:c>
+      <x:c r="C16" s="38" t="str">
+        <x:v>men</x:v>
+      </x:c>
+      <x:c r="D16" s="38" t="str">
+        <x:v>road</x:v>
+      </x:c>
+      <x:c r="E16" s="83" t="n">
+        <x:v>14999</x:v>
+      </x:c>
+      <x:c r="F16" s="83" t="n">
+        <x:v>19999</x:v>
+      </x:c>
+      <x:c r="G16" s="38" t="str">
+        <x:v>https://in.puma.com/in/en/sports/sports-running/nitro-collection</x:v>
+      </x:c>
+      <x:c r="H16" s="38" t="str">
+        <x:v>candidate</x:v>
+      </x:c>
+      <x:c r="I16" s="86" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="J16" s="38" t="str">
+        <x:f>IF(H16="already_in_catalog","Compare price and source","Open product page; complete specs")</x:f>
+        <x:v>Open product page; complete specs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="38" t="str">
+        <x:v>PUMA</x:v>
+      </x:c>
+      <x:c r="B17" s="38" t="str">
+        <x:v>Deviate Pure NITRO</x:v>
+      </x:c>
+      <x:c r="C17" s="38" t="str">
+        <x:v>men</x:v>
+      </x:c>
+      <x:c r="D17" s="38" t="str">
+        <x:v>road</x:v>
+      </x:c>
+      <x:c r="E17" s="83" t="n">
+        <x:v>14999</x:v>
+      </x:c>
+      <x:c r="F17" s="83" t="n">
+        <x:v>14999</x:v>
+      </x:c>
+      <x:c r="G17" s="38" t="str">
+        <x:v>https://in.puma.com/in/en/sports/sports-running/nitro-collection</x:v>
+      </x:c>
+      <x:c r="H17" s="38" t="str">
+        <x:v>candidate</x:v>
+      </x:c>
+      <x:c r="I17" s="86" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="J17" s="38" t="str">
+        <x:f>IF(H17="already_in_catalog","Compare price and source","Open product page; complete specs")</x:f>
+        <x:v>Open product page; complete specs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="38" t="str">
+        <x:v>PUMA</x:v>
+      </x:c>
+      <x:c r="B18" s="38" t="str">
+        <x:v>ForeverRun NITRO 2</x:v>
+      </x:c>
+      <x:c r="C18" s="38" t="str">
+        <x:v>men</x:v>
+      </x:c>
+      <x:c r="D18" s="38" t="str">
+        <x:v>road</x:v>
+      </x:c>
+      <x:c r="E18" s="83" t="n">
+        <x:v>10499</x:v>
+      </x:c>
+      <x:c r="F18" s="83" t="n">
+        <x:v>14999</x:v>
+      </x:c>
+      <x:c r="G18" s="38" t="str">
+        <x:v>https://in.puma.com/in/en/sports/sports-running/nitro-collection</x:v>
+      </x:c>
+      <x:c r="H18" s="38" t="str">
+        <x:v>candidate</x:v>
+      </x:c>
+      <x:c r="I18" s="86" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="J18" s="38" t="str">
+        <x:f>IF(H18="already_in_catalog","Compare price and source","Open product page; complete specs")</x:f>
+        <x:v>Open product page; complete specs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="38" t="str">
+        <x:v>PUMA</x:v>
+      </x:c>
+      <x:c r="B19" s="38" t="str">
+        <x:v>Propio NITRO</x:v>
+      </x:c>
+      <x:c r="C19" s="38" t="str">
+        <x:v>men</x:v>
+      </x:c>
+      <x:c r="D19" s="38" t="str">
+        <x:v>road</x:v>
+      </x:c>
+      <x:c r="E19" s="83" t="n">
+        <x:v>6599</x:v>
+      </x:c>
+      <x:c r="F19" s="83" t="n">
+        <x:v>10999</x:v>
+      </x:c>
+      <x:c r="G19" s="38" t="str">
+        <x:v>https://in.puma.com/in/en/sports/sports-running/nitro-collection</x:v>
+      </x:c>
+      <x:c r="H19" s="38" t="str">
+        <x:v>candidate</x:v>
+      </x:c>
+      <x:c r="I19" s="86" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="J19" s="38" t="str">
+        <x:f>IF(H19="already_in_catalog","Compare price and source","Open product page; complete specs")</x:f>
+        <x:v>Open product page; complete specs</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="38" t="str">
+        <x:v>PUMA</x:v>
+      </x:c>
+      <x:c r="B20" s="38" t="str">
+        <x:v>Magnify NITRO 3</x:v>
+      </x:c>
+      <x:c r="C20" s="38" t="str">
+        <x:v>men</x:v>
+      </x:c>
+      <x:c r="D20" s="38" t="str">
+        <x:v>road</x:v>
+      </x:c>
+      <x:c r="E20" s="83" t="n">
+        <x:v>9749</x:v>
+      </x:c>
+      <x:c r="F20" s="83" t="n">
+        <x:v>14999</x:v>
+      </x:c>
+      <x:c r="G20" s="38" t="str">
+        <x:v>https://in.puma.com/in/en/sports/sports-running/nitro-collection</x:v>
+      </x:c>
+      <x:c r="H20" s="38" t="str">
+        <x:v>already_in_catalog</x:v>
+      </x:c>
+      <x:c r="I20" s="86" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="J20" s="38" t="str">
+        <x:f>IF(H20="already_in_catalog","Compare price and source","Open product page; complete specs")</x:f>
+        <x:v>Compare price and source</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="38" t="str">
+        <x:v>PUMA</x:v>
+      </x:c>
+      <x:c r="B21" s="38" t="str">
+        <x:v>Deviate NITRO 4</x:v>
+      </x:c>
+      <x:c r="C21" s="38" t="str">
+        <x:v>men</x:v>
+      </x:c>
+      <x:c r="D21" s="38" t="str">
+        <x:v>road</x:v>
+      </x:c>
+      <x:c r="E21" s="83" t="n">
+        <x:v>16999</x:v>
+      </x:c>
+      <x:c r="F21" s="83" t="n">
+        <x:v>16999</x:v>
+      </x:c>
+      <x:c r="G21" s="38" t="str">
+        <x:v>https://in.puma.com/in/en/sports/sports-running/nitro-collection</x:v>
+      </x:c>
+      <x:c r="H21" s="38" t="str">
+        <x:v>already_in_catalog</x:v>
+      </x:c>
+      <x:c r="I21" s="86" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="J21" s="38" t="str">
+        <x:f>IF(H21="already_in_catalog","Compare price and source","Open product page; complete specs")</x:f>
+        <x:v>Compare price and source</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22">
+      <x:c r="A22" s="39" t="str">
+        <x:v>PUMA</x:v>
+      </x:c>
+      <x:c r="B22" s="39" t="str">
+        <x:v>Deviate NITRO Elite 4</x:v>
+      </x:c>
+      <x:c r="C22" s="39" t="str">
+        <x:v>men</x:v>
+      </x:c>
+      <x:c r="D22" s="39" t="str">
+        <x:v>road</x:v>
+      </x:c>
+      <x:c r="E22" s="84" t="n">
+        <x:v>21999</x:v>
+      </x:c>
+      <x:c r="F22" s="84" t="n">
+        <x:v>21999</x:v>
+      </x:c>
+      <x:c r="G22" s="39" t="str">
+        <x:v>https://in.puma.com/in/en/sports/sports-running/nitro-collection</x:v>
+      </x:c>
+      <x:c r="H22" s="39" t="str">
+        <x:v>already_in_catalog</x:v>
+      </x:c>
+      <x:c r="I22" s="87" t="str">
+        <x:v>2026-07-30</x:v>
+      </x:c>
+      <x:c r="J22" s="39" t="str">
+        <x:f>IF(H22="already_in_catalog","Compare price and source","Open product page; complete specs")</x:f>
+        <x:v>Compare price and source</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:J1"/>
+    <x:mergeCell ref="A2:J2"/>
+  </x:mergeCells>
+  <x:conditionalFormatting sqref="H5:H22">
+    <x:cfRule type="containsText" dxfId="3" priority="1" operator="containsText" text="already_in_catalog"/>
+    <x:cfRule type="containsText" dxfId="4" priority="2" operator="containsText" text="candidate"/>
+  </x:conditionalFormatting>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>